<commit_message>
add a loading ui and the prompt
</commit_message>
<xml_diff>
--- a/model/Model Records.xlsx
+++ b/model/Model Records.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\taro\model\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\tarot\model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C58DD977-0FD8-4211-8BC2-8404D39A64AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F76DCCBB-9164-46F4-9506-CE436946F2AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2362D553-DFEC-458D-9744-BC2A5A97024A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{2362D553-DFEC-458D-9744-BC2A5A97024A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Model modification" sheetId="3" r:id="rId2"/>
+    <sheet name="To-do in the future" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="66">
   <si>
     <t>Model name</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -240,6 +242,675 @@
   </si>
   <si>
     <t>to automatically register a service worker, and tell a browser that this is a PWA</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>taro_app_11</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>add the function of "google analynatics"</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>inject GA at the top of the codes</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fix the path for the images</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">No!
+Spent hours.
+Put it aside now since there are only a few users.(Priority ↓) </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>To do list in the future</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. add the function of "google analynatics"</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Reason</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>entering the website becomes slower after applying this function</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>delete codes related to GA function</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>return to taro_app_10, (change the setting on render)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Note</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>I didn't do it because I just ran the taro_app_10 version and let this version alone.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Found</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. 3.45 dollars today 2025/11/5 openai api</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>11月2号星期日开始发出去的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">change the prompt and parameters
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>你是一位灵性而深具洞察的塔罗牌大师，融合荣格心理学、象征学与神秘学的理解，亦熟悉人性的阴影面与社会现实中的复杂动因。你既能温柔地陪伴，也能直面潜藏的欲望、恐惧与防御机制，帮助咨询者看清内在冲突与外在局势。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>请用优雅而自然的语言解读牌义，不使用列表或编号，而是用段落叙事的方式展开。语气自然流动，像在静谧空间中轻声对话，但不回避人性的复杂性。你可以适度揭示可能的操控、逃避、欲望、权力斗争等心理动因，不批判，只映照。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>每次解读分为三个层次：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>）一句直觉性的判断或建议；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>）【灵性与心理解读】——</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>描述牌象意象，结合心理层面与能量流动，讲述问题背后的内在状态与成长方向，并指出可能的心理盲点或潜在风险；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>）给出现实生活中的小行动或心态转化方式，并以一句温暖而真实的“塔罗祝语”收尾。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+temperature=0.85, presence_penalty=0.8, frequency_penalty=0.5,</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Response to feedback No.3 (I have same feeling)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">change the prompt:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>你是一位灵性而深具洞察的塔罗牌大师，融合荣格心理学、象征学与神秘学的理解，亦熟悉人性的阴影面与社会现实中的复杂动因。你既能温柔地陪伴，也能在面对现实抉择时，提供清晰而深刻的洞察。你擅长在模糊与矛盾中辨识能量流动的倾向，帮助咨询者看清不同选项背后的心理动因与可能走向。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>请用优雅而自然的语言解读牌义，不使用列表或编号，而是用段落叙事的方式展开。语气自然流动，像在静谧空间中轻声对话，但不回避人性的复杂性。你可以适度揭示可能的操控、逃避、欲望、权力斗争等心理动因，不批判，只映照。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>每次解读分为三个层次：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>）一句直觉性的判断或建议；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>）【灵性与心理解读】——</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>描述牌象意象，结合心理层面与能量流动，讲述问题背后的内在状态与成长方向，并指出可能的心理盲点或潜在风险；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>）给出现实生活中的小行动或心态转化方式，并以一句温暖而真实的“塔罗祝语”收尾。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>如果问题是两个方案的选择，请：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>分别描述两个选项的能量象征与心理动因；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>指出每个选项可能带来的成长方向与挑战；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>结合牌面能量，给出你感受到的倾向性建议（但不强迫决定）；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>最后仍以一句温暖的“塔罗祝语”收尾，鼓励咨询者在觉察中做出选择。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>请避免空泛的“</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>follow your heart”</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>式建议，除非牌面明确指向内在觉醒。若咨询者尚未觉察内心，请帮助他们识别内在冲突、惯性、恐惧或欲望的来源，使他们更有力量做出选择。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Response to feedback No.2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Response to feedback No.12 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>taro_app_12</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>taro_app_10</t>
+  </si>
+  <si>
+    <t>详情在model modification</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. add the loading ui
+2. add spread explanation(三张是过去未来和现在，6张是对应过去、现在、未来、原因、环境、对策)
+3.add prompt 
+-如用户抽了三张牌，第1张，第2张，第3张分别代表过去、未来、现在
+-如用户抽了六张牌，第1张到第6张依此代表过去、现在、未来、原因、环境、对策</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>add the prompt</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">
+请注意以下几点以增强解读的真实感与可信度：
+- 在解读中适度展现你是如何从牌面意象、位置、组合中推导出判断的，让咨询者感受到你的思考轨迹；
+- 保持牌面之间的内在逻辑一致性，避免彼此矛盾的解读，可指出牌面之间的张力、呼应或对比；（后两句没加）
+- 你可以适度提出共情式问题，引导咨询者自我觉察，例如：“你是否曾因为害怕失去而迟迟不敢行动？”
+- 你是一位温柔、诚实、略带神秘气质的塔罗师，风格稳定，语言中常带有自然意象与心理洞察。请保持一致的表达风格与人格特质。</t>
+    </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -247,7 +918,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -292,6 +963,42 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Microsoft YaHei UI"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0" tint="-0.499984740745262"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0" tint="-0.499984740745262"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -301,7 +1008,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -509,13 +1216,63 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="2" tint="-0.24994659260841701"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2" tint="-0.24994659260841701"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2" tint="-0.24994659260841701"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2" tint="-0.24994659260841701"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2" tint="-0.24994659260841701"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="2" tint="-0.24994659260841701"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2" tint="-0.24994659260841701"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2" tint="-0.24994659260841701"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="2" tint="-0.24994659260841701"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -567,9 +1324,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -581,6 +1335,51 @@
     </xf>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -916,7 +1715,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4CDA32B-5715-4694-9741-2DB3D4B4CE16}">
-  <dimension ref="B3:H27"/>
+  <dimension ref="B3:I28"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -924,13 +1723,14 @@
     <col min="3" max="3" width="18.6640625" customWidth="1"/>
     <col min="4" max="4" width="55.44140625" customWidth="1"/>
     <col min="5" max="5" width="47.77734375" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="16.44140625" customWidth="1"/>
-    <col min="8" max="8" width="38.6640625" customWidth="1"/>
+    <col min="6" max="6" width="18.44140625" customWidth="1"/>
+    <col min="7" max="7" width="12.44140625" customWidth="1"/>
+    <col min="8" max="8" width="16.44140625" customWidth="1"/>
+    <col min="9" max="9" width="38.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:8" ht="14.4" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="2:8" ht="21" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:9" ht="14.4" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="2:9" ht="21" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
@@ -946,12 +1746,13 @@
       <c r="F4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="23"/>
+      <c r="H4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H4" s="2"/>
-    </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I4" s="2"/>
+    </row>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="6">
         <v>1</v>
       </c>
@@ -963,12 +1764,13 @@
       <c r="F5" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="24"/>
+      <c r="H5" s="8">
         <v>45959</v>
       </c>
-      <c r="H5" s="2"/>
-    </row>
-    <row r="6" spans="2:8" ht="41.4" x14ac:dyDescent="0.25">
+      <c r="I5" s="2"/>
+    </row>
+    <row r="6" spans="2:9" ht="41.4" x14ac:dyDescent="0.25">
       <c r="B6" s="6">
         <v>2</v>
       </c>
@@ -984,13 +1786,14 @@
       <c r="F6" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="24"/>
+      <c r="H6" s="8">
         <v>45959</v>
       </c>
-      <c r="H6" s="2"/>
-    </row>
-    <row r="7" spans="2:8" ht="41.4" x14ac:dyDescent="0.25">
-      <c r="B7" s="10">
+      <c r="I6" s="2"/>
+    </row>
+    <row r="7" spans="2:9" ht="41.4" x14ac:dyDescent="0.25">
+      <c r="B7" s="6">
         <v>3</v>
       </c>
       <c r="C7" s="7" t="s">
@@ -1005,13 +1808,16 @@
       <c r="F7" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G7" s="24"/>
+      <c r="H7" s="8">
         <v>45960</v>
       </c>
-      <c r="H7" s="2"/>
-    </row>
-    <row r="8" spans="2:8" ht="41.4" x14ac:dyDescent="0.25">
-      <c r="B8" s="10"/>
+      <c r="I7" s="2"/>
+    </row>
+    <row r="8" spans="2:9" ht="41.4" x14ac:dyDescent="0.25">
+      <c r="B8" s="6">
+        <v>4</v>
+      </c>
       <c r="C8" s="7" t="s">
         <v>14</v>
       </c>
@@ -1024,13 +1830,16 @@
       <c r="F8" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="25"/>
+      <c r="H8" s="8">
         <v>45960</v>
       </c>
-      <c r="H8" s="2"/>
-    </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="10"/>
+      <c r="I8" s="2"/>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B9" s="6">
+        <v>5</v>
+      </c>
       <c r="C9" s="7" t="s">
         <v>18</v>
       </c>
@@ -1043,13 +1852,16 @@
       <c r="F9" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="25"/>
+      <c r="H9" s="8">
         <v>45960</v>
       </c>
-      <c r="H9" s="2"/>
-    </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B10" s="10"/>
+      <c r="I9" s="2"/>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B10" s="6">
+        <v>6</v>
+      </c>
       <c r="C10" s="7" t="s">
         <v>17</v>
       </c>
@@ -1062,13 +1874,16 @@
       <c r="F10" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="25"/>
+      <c r="H10" s="8">
         <v>45960</v>
       </c>
-      <c r="H10" s="2"/>
-    </row>
-    <row r="11" spans="2:8" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="B11" s="10"/>
+      <c r="I10" s="2"/>
+    </row>
+    <row r="11" spans="2:9" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="B11" s="6">
+        <v>7</v>
+      </c>
       <c r="C11" s="7" t="s">
         <v>21</v>
       </c>
@@ -1079,12 +1894,15 @@
         <v>23</v>
       </c>
       <c r="F11" s="14"/>
-      <c r="G11" s="8">
+      <c r="G11" s="25"/>
+      <c r="H11" s="8">
         <v>45960</v>
       </c>
     </row>
-    <row r="12" spans="2:8" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="B12" s="10"/>
+    <row r="12" spans="2:9" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="B12" s="6">
+        <v>8</v>
+      </c>
       <c r="C12" s="7" t="s">
         <v>24</v>
       </c>
@@ -1097,12 +1915,15 @@
       <c r="F12" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="G12" s="8">
+      <c r="G12" s="25"/>
+      <c r="H12" s="8">
         <v>45961</v>
       </c>
     </row>
-    <row r="13" spans="2:8" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="B13" s="10"/>
+    <row r="13" spans="2:9" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="B13" s="6">
+        <v>9</v>
+      </c>
       <c r="C13" s="7" t="s">
         <v>27</v>
       </c>
@@ -1113,15 +1934,18 @@
       <c r="F13" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="G13" s="8">
+      <c r="G13" s="25"/>
+      <c r="H13" s="8">
         <v>45961</v>
       </c>
-      <c r="H13" s="17" t="s">
+      <c r="I13" s="21" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="2:8" ht="55.2" x14ac:dyDescent="0.25">
-      <c r="B14" s="10"/>
+    <row r="14" spans="2:9" ht="55.2" x14ac:dyDescent="0.25">
+      <c r="B14" s="6">
+        <v>10</v>
+      </c>
       <c r="C14" s="7" t="s">
         <v>29</v>
       </c>
@@ -1134,16 +1958,19 @@
       <c r="F14" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="G14" s="8">
+      <c r="G14" s="25"/>
+      <c r="H14" s="8">
         <v>45962</v>
       </c>
-      <c r="H14" s="18" t="s">
+      <c r="I14" s="21" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B15" s="19"/>
-      <c r="C15" s="20" t="s">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B15" s="6">
+        <v>11</v>
+      </c>
+      <c r="C15" s="19" t="s">
         <v>35</v>
       </c>
       <c r="D15" s="14"/>
@@ -1153,14 +1980,17 @@
       <c r="F15" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="G15" s="8">
+      <c r="G15" s="25"/>
+      <c r="H15" s="8">
         <v>45963</v>
       </c>
-      <c r="H15" s="18"/>
-    </row>
-    <row r="16" spans="2:8" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="B16" s="19"/>
-      <c r="C16" s="20" t="s">
+      <c r="I15" s="17"/>
+    </row>
+    <row r="16" spans="2:9" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="B16" s="6">
+        <v>12</v>
+      </c>
+      <c r="C16" s="19" t="s">
         <v>37</v>
       </c>
       <c r="D16" s="14" t="s">
@@ -1169,59 +1999,372 @@
       <c r="E16" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="F16" s="20" t="s">
+      <c r="F16" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="G16" s="21"/>
-      <c r="H16" s="18"/>
-    </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B17" s="19"/>
-      <c r="C17" s="20"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="8">
+        <v>45963</v>
+      </c>
+      <c r="I16" s="17"/>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B17" s="6">
+        <v>13</v>
+      </c>
+      <c r="C17" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="D17" s="14"/>
+      <c r="E17" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="F17" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="G17" s="26"/>
+      <c r="H17" s="8">
+        <v>45963</v>
+      </c>
+      <c r="I17" s="17"/>
+    </row>
+    <row r="18" spans="2:9" ht="69" x14ac:dyDescent="0.25">
+      <c r="B18" s="28">
+        <v>14</v>
+      </c>
+      <c r="C18" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="D18" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="E18" s="30" t="s">
+        <v>41</v>
+      </c>
+      <c r="F18" s="29" t="s">
+        <v>37</v>
+      </c>
+      <c r="G18" s="31" t="s">
+        <v>50</v>
+      </c>
+      <c r="H18" s="32">
+        <v>45964</v>
+      </c>
+      <c r="I18" s="21" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B19" s="6">
+        <v>15</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="D19" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="E19" s="14"/>
+      <c r="F19" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="G19" s="27"/>
+      <c r="H19" s="20"/>
+      <c r="I19" s="17"/>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B20" s="6">
+        <v>16</v>
+      </c>
+      <c r="C20" s="19"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="20"/>
+      <c r="I20" s="17"/>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B21" s="6">
+        <v>17</v>
+      </c>
+      <c r="C21" s="19"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="27"/>
+      <c r="H21" s="20"/>
+      <c r="I21" s="17"/>
+    </row>
+    <row r="22" spans="2:9" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="11"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="13"/>
+      <c r="H22" s="13"/>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D28" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA669490-90C1-4BC3-89F7-B5C17A6F4FB6}">
+  <dimension ref="B3:G22"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="6" style="1" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" customWidth="1"/>
+    <col min="4" max="4" width="75.6640625" customWidth="1"/>
+    <col min="5" max="5" width="60.88671875" customWidth="1"/>
+    <col min="6" max="6" width="16.44140625" customWidth="1"/>
+    <col min="7" max="7" width="38.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:7" ht="14.4" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="2:7" ht="21" x14ac:dyDescent="0.25">
+      <c r="B4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" ht="41.4" x14ac:dyDescent="0.25">
+      <c r="B5" s="6">
+        <v>1</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="F5" s="34">
+        <v>45965</v>
+      </c>
+      <c r="G5" s="33" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" ht="241.8" x14ac:dyDescent="0.25">
+      <c r="B6" s="6">
+        <v>2</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F6" s="9"/>
+      <c r="G6" s="33"/>
+    </row>
+    <row r="7" spans="2:7" ht="385.8" x14ac:dyDescent="0.25">
+      <c r="B7" s="10">
+        <v>3</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="F7" s="9"/>
+      <c r="G7" s="33"/>
+    </row>
+    <row r="8" spans="2:7" ht="158.4" x14ac:dyDescent="0.25">
+      <c r="B8" s="10"/>
+      <c r="C8" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="35" t="s">
+        <v>65</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="F8" s="14"/>
+      <c r="G8" s="33"/>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B9" s="10"/>
+      <c r="C9" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="33"/>
+    </row>
+    <row r="10" spans="2:7" ht="82.8" x14ac:dyDescent="0.25">
+      <c r="B10" s="10"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="33"/>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B11" s="10"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="33"/>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B12" s="10"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="14"/>
+      <c r="G12" s="33"/>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B13" s="10"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="14"/>
+      <c r="G13" s="33"/>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B14" s="10"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="33"/>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B15" s="18"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="33"/>
+    </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B16" s="18"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="33"/>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="18"/>
+      <c r="C17" s="19"/>
       <c r="D17" s="14"/>
       <c r="E17" s="14"/>
       <c r="F17" s="14"/>
-      <c r="G17" s="21"/>
-      <c r="H17" s="18"/>
-    </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B18" s="19"/>
-      <c r="C18" s="20"/>
+      <c r="G17" s="33"/>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B18" s="18"/>
+      <c r="C18" s="19"/>
       <c r="D18" s="14"/>
       <c r="E18" s="14"/>
       <c r="F18" s="14"/>
-      <c r="G18" s="21"/>
-      <c r="H18" s="18"/>
-    </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B19" s="19"/>
-      <c r="C19" s="20"/>
+      <c r="G18" s="33"/>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B19" s="18"/>
+      <c r="C19" s="19"/>
       <c r="D19" s="14"/>
       <c r="E19" s="14"/>
       <c r="F19" s="14"/>
-      <c r="G19" s="21"/>
-      <c r="H19" s="18"/>
-    </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B20" s="19"/>
-      <c r="C20" s="20"/>
+      <c r="G19" s="33"/>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B20" s="18"/>
+      <c r="C20" s="19"/>
       <c r="D20" s="14"/>
       <c r="E20" s="14"/>
       <c r="F20" s="14"/>
-      <c r="G20" s="21"/>
-      <c r="H20" s="18"/>
-    </row>
-    <row r="21" spans="2:8" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="11"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="16"/>
-      <c r="G21" s="13"/>
-    </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="D27" t="s">
-        <v>33</v>
+      <c r="G20" s="33"/>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B21" s="18"/>
+      <c r="C21" s="19"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="33"/>
+    </row>
+    <row r="22" spans="2:7" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="11"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="13"/>
+      <c r="G22" s="33"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CAC97C2-8F2F-4876-9208-CADAE372E0B5}">
+  <dimension ref="B3:F4"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="47.33203125" customWidth="1"/>
+    <col min="5" max="5" width="40.44140625" customWidth="1"/>
+    <col min="6" max="6" width="27.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:6" ht="15.6" x14ac:dyDescent="0.25">
+      <c r="B3" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" ht="15.6" x14ac:dyDescent="0.25">
+      <c r="B4" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="E4" t="s">
+        <v>54</v>
+      </c>
+      <c r="F4" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add two models tarot_app_13.py and tarot_app_14.py, and use the latter one
</commit_message>
<xml_diff>
--- a/model/Model Records.xlsx
+++ b/model/Model Records.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\tarot\model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F76DCCBB-9164-46F4-9506-CE436946F2AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7BEA356-C881-492A-84E0-DF2E00394325}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{2362D553-DFEC-458D-9744-BC2A5A97024A}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="92">
   <si>
     <t>Model name</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -860,10 +860,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Response to feedback No.2</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t xml:space="preserve">Response to feedback No.12 </t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -876,14 +872,6 @@
   </si>
   <si>
     <t>详情在model modification</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1. add the loading ui
-2. add spread explanation(三张是过去未来和现在，6张是对应过去、现在、未来、原因、环境、对策)
-3.add prompt 
--如用户抽了三张牌，第1张，第2张，第3张分别代表过去、未来、现在
--如用户抽了六张牌，第1张到第6张依此代表过去、现在、未来、原因、环境、对策</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -913,23 +901,275 @@
     </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>11日5日发pyq</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>1. add the loading ui
+2. add spread explanation</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>(三张是过去未来和现在，6张是对应过去、现在、未来、原因、环境、对策)
+3.add prompt 
+-如用户抽了三张牌，第1张，第2张，第3张分别代表过去、未来、现在
+-如用户抽了六张牌，第1张到第6张依此代表过去、现在、未来、原因、环境、对策</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. change the prompt of the first sentence. Please be straightforward. (Action needed: Understand the structured prompt and determine if it clarifies the vaguely expressed question in the text.)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>1.change the prompt:
+你是一位经验丰富、温柔理性的塔罗大师：无论用户抽到哪一张牌（或逆位），你的回答都应包含以下结构与风格：
+1.开场吁应问题（如“针对你一．的问题，抽到．一，这是一个值得注意的信号”）
+说明牌面含义（分条解释）
+2.针对问题进行具体分析，指出可能性高低与原因
+3.给出“塔罗提醒”与“塔罗建议”，风格带有温柔引导
+4.最后用“结论”收尾，结构清晰、逻辑自然
+5.适当使用表情符号（</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Emoji"/>
+        <family val="3"/>
+      </rPr>
+      <t>⚠️</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="3"/>
+      </rPr>
+      <t>📉</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="3"/>
+      </rPr>
+      <t>🐌</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="3"/>
+      </rPr>
+      <t>💡</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="3"/>
+      </rPr>
+      <t>📊</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 等)，语气中带一点占卜神秘感与现实建议的平衡
+输出语言为中文：
+现在请根据用户的问题和抽到的牌进行解读：
+temperature=0.8, presence_penalty=0.6, frequency_penalty=0.3</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>taro_app_12</t>
+  </si>
+  <si>
+    <t>taro_app_13</t>
+  </si>
+  <si>
+    <t>要点了生成解读之后再出现补充信息，要点了补充信息之后再出现完整对话</t>
+  </si>
+  <si>
+    <t>Response to feedback No.2</t>
+  </si>
+  <si>
+    <t>Response to feedback No.5</t>
+  </si>
+  <si>
+    <t>Response to feedback No.7</t>
+  </si>
+  <si>
+    <t>文本框上面说明内容：如想对占卜的问题继续问</t>
+  </si>
+  <si>
+    <t>Response to feedback No.9</t>
+  </si>
+  <si>
+    <t>把牌阵删到两个</t>
+  </si>
+  <si>
+    <t>Response to feedback No.19</t>
+  </si>
+  <si>
+    <t>Response to feedback No.24</t>
+  </si>
+  <si>
+    <t>只留三张和单张牌阵</t>
+  </si>
+  <si>
+    <t>Response to feedback No.25</t>
+  </si>
+  <si>
+    <t>把单张牌的推荐语直接改成“推荐”。
+删掉10张牌 3张和6张。
+写在前面，内心的指引。</t>
+  </si>
+  <si>
+    <t>圣杯侍从未找到牌图“page_of_cups.jpg”
+pages_of_cups因为图的名字多了一个s。应该是page</t>
+  </si>
+  <si>
+    <t>Response to feedback No.26</t>
+  </si>
+  <si>
+    <t>Response to feedback No.27</t>
+  </si>
+  <si>
+    <t>把私人命理师改成灵枢</t>
+  </si>
+  <si>
+    <t>设置一个按钮 重新占卜  （抽完一张牌 之后 怎么再来一次？
+由于不能清空输入文字，于是不要了。直接教人重新刷新页面</t>
+  </si>
+  <si>
+    <t>在页面加上：
+灵枢旨在提供引导，帮助深度的自我洞察，而非重复验证已知答案。建议在心境澄明时进行，并着重于对结果的反思而非结果本身
+· 帮助人理解自己
+· 提供精神空间
+· 减轻痛苦
+· 帮忙看到盲点
+同一问题一周内不建议重复问（最终决定只要了这一个句话。面对公众，内容会变得稀薄）
+灵枢希望你先觉察今天的心情与状况，再决定是否继续追问。
+你的心，其实已经给了你答案。
+灵枢希望陪伴您探索内心，而不是反复验证已知的答案。（写了）</t>
+  </si>
+  <si>
+    <t>用户点一个按钮：
+「我需要一个明确判断」
+以此得到两个类型占卜
+用户选择模式（UI）
+「指引型解读」
+「决策型解读」
+只要用户点了第二个，就切 system prompt。</t>
+  </si>
+  <si>
+    <t>taro_app_14</t>
+  </si>
+  <si>
+    <t>model14</t>
+  </si>
+  <si>
+    <t>model13</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="等线"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -958,7 +1198,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Aptos Narrow"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -980,7 +1220,7 @@
       <b/>
       <sz val="11"/>
       <color theme="0" tint="-0.499984740745262"/>
-      <name val="等线"/>
+      <name val="Aptos Narrow"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -998,6 +1238,35 @@
       <name val="宋体"/>
       <family val="3"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI Emoji"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI Symbol"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1272,7 +1541,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1381,9 +1650,18 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1399,7 +1677,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1716,7 +1994,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4CDA32B-5715-4694-9741-2DB3D4B4CE16}">
   <dimension ref="B3:I28"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="6" style="1" customWidth="1"/>
@@ -1729,7 +2007,7 @@
     <col min="9" max="9" width="38.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:9" ht="14.4" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="2:9" ht="21" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
         <v>7</v>
@@ -1814,7 +2092,7 @@
       </c>
       <c r="I7" s="2"/>
     </row>
-    <row r="8" spans="2:9" ht="41.4" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:9" ht="57.6" x14ac:dyDescent="0.25">
       <c r="B8" s="6">
         <v>4</v>
       </c>
@@ -1880,7 +2158,7 @@
       </c>
       <c r="I10" s="2"/>
     </row>
-    <row r="11" spans="2:9" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:9" ht="28.8" x14ac:dyDescent="0.25">
       <c r="B11" s="6">
         <v>7</v>
       </c>
@@ -1899,7 +2177,7 @@
         <v>45960</v>
       </c>
     </row>
-    <row r="12" spans="2:9" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:9" ht="28.8" x14ac:dyDescent="0.25">
       <c r="B12" s="6">
         <v>8</v>
       </c>
@@ -1942,7 +2220,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="2:9" ht="55.2" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:9" ht="57.6" x14ac:dyDescent="0.25">
       <c r="B14" s="6">
         <v>10</v>
       </c>
@@ -1986,7 +2264,7 @@
       </c>
       <c r="I15" s="17"/>
     </row>
-    <row r="16" spans="2:9" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:9" ht="43.2" x14ac:dyDescent="0.25">
       <c r="B16" s="6">
         <v>12</v>
       </c>
@@ -2059,44 +2337,62 @@
         <v>15</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E19" s="14"/>
       <c r="F19" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G19" s="27"/>
-      <c r="H19" s="20"/>
+      <c r="H19" s="8">
+        <v>45968</v>
+      </c>
       <c r="I19" s="17"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B20" s="6">
         <v>16</v>
       </c>
-      <c r="C20" s="19"/>
-      <c r="D20" s="14"/>
+      <c r="C20" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>62</v>
+      </c>
       <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
+      <c r="F20" s="19" t="s">
+        <v>60</v>
+      </c>
       <c r="G20" s="27"/>
-      <c r="H20" s="20"/>
+      <c r="H20" s="20">
+        <v>46020</v>
+      </c>
       <c r="I20" s="17"/>
     </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:9" ht="144" x14ac:dyDescent="0.25">
       <c r="B21" s="6">
         <v>17</v>
       </c>
-      <c r="C21" s="19"/>
-      <c r="D21" s="14"/>
+      <c r="C21" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>88</v>
+      </c>
       <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
+      <c r="F21" s="19" t="s">
+        <v>69</v>
+      </c>
       <c r="G21" s="27"/>
-      <c r="H21" s="20"/>
+      <c r="H21" s="20">
+        <v>46020</v>
+      </c>
       <c r="I21" s="17"/>
     </row>
-    <row r="22" spans="2:9" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="11"/>
       <c r="C22" s="12"/>
       <c r="D22" s="12"/>
@@ -2118,8 +2414,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA669490-90C1-4BC3-89F7-B5C17A6F4FB6}">
-  <dimension ref="B3:G22"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <dimension ref="B3:G23"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="6" style="1" customWidth="1"/>
@@ -2130,7 +2426,7 @@
     <col min="7" max="7" width="38.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:7" ht="14.4" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="2:7" ht="21" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
         <v>7</v>
@@ -2171,12 +2467,12 @@
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="2:7" ht="241.8" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:7" ht="256.2" x14ac:dyDescent="0.25">
       <c r="B6" s="6">
         <v>2</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D6" s="9" t="s">
         <v>56</v>
@@ -2184,153 +2480,256 @@
       <c r="E6" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="F6" s="9"/>
+      <c r="F6" s="34">
+        <v>45968</v>
+      </c>
       <c r="G6" s="33"/>
     </row>
-    <row r="7" spans="2:7" ht="385.8" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:7" ht="400.2" x14ac:dyDescent="0.25">
       <c r="B7" s="10">
         <v>3</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>58</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="F7" s="9"/>
+        <v>59</v>
+      </c>
+      <c r="F7" s="34">
+        <v>45968</v>
+      </c>
       <c r="G7" s="33"/>
     </row>
-    <row r="8" spans="2:7" ht="158.4" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:7" ht="216" x14ac:dyDescent="0.25">
       <c r="B8" s="10"/>
       <c r="C8" s="7" t="s">
         <v>37</v>
       </c>
       <c r="D8" s="35" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="F8" s="14"/>
+        <v>71</v>
+      </c>
+      <c r="F8" s="34">
+        <v>45968</v>
+      </c>
       <c r="G8" s="33"/>
     </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:7" ht="114" x14ac:dyDescent="0.25">
       <c r="B9" s="10"/>
       <c r="C9" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
+      </c>
+      <c r="D9" s="36" t="s">
+        <v>65</v>
       </c>
       <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
+      <c r="F9" s="34">
+        <v>45968</v>
+      </c>
       <c r="G9" s="33"/>
     </row>
-    <row r="10" spans="2:7" ht="82.8" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:7" ht="41.4" x14ac:dyDescent="0.25">
       <c r="B10" s="10"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="14" t="s">
-        <v>64</v>
+      <c r="C10" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10" s="37" t="s">
+        <v>66</v>
       </c>
       <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
+      <c r="F10" s="34">
+        <v>45968</v>
+      </c>
       <c r="G10" s="33"/>
     </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:7" ht="204" x14ac:dyDescent="0.25">
       <c r="B11" s="10"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="14"/>
+      <c r="C11" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>67</v>
+      </c>
       <c r="E11" s="14"/>
       <c r="F11" s="14"/>
       <c r="G11" s="33"/>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B12" s="10"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="33"/>
-    </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C12" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="F12" s="20">
+        <v>46020</v>
+      </c>
+      <c r="G12" s="33" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" ht="28.8" x14ac:dyDescent="0.25">
       <c r="B13" s="10"/>
       <c r="C13" s="7"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="33"/>
+      <c r="D13" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="F13" s="20">
+        <v>46020</v>
+      </c>
+      <c r="G13" s="33" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B14" s="10"/>
       <c r="C14" s="7"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="33"/>
+      <c r="D14" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="F14" s="20">
+        <v>46020</v>
+      </c>
+      <c r="G14" s="33" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B15" s="18"/>
       <c r="C15" s="19"/>
-      <c r="D15" s="14"/>
+      <c r="D15" s="14" t="s">
+        <v>76</v>
+      </c>
       <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="33"/>
-    </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F15" s="20">
+        <v>46020</v>
+      </c>
+      <c r="G15" s="33" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7" ht="187.2" x14ac:dyDescent="0.25">
       <c r="B16" s="18"/>
       <c r="C16" s="19"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="33"/>
+      <c r="D16" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="F16" s="20">
+        <v>46020</v>
+      </c>
+      <c r="G16" s="33" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="18"/>
       <c r="C17" s="19"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="33"/>
+      <c r="D17" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="E17" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="F17" s="20">
+        <v>46020</v>
+      </c>
+      <c r="G17" s="33" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="18"/>
       <c r="C18" s="19"/>
       <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
       <c r="G18" s="33"/>
     </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:7" ht="43.2" x14ac:dyDescent="0.25">
       <c r="B19" s="18"/>
       <c r="C19" s="19"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="33"/>
-    </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D19" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="F19" s="20">
+        <v>46020</v>
+      </c>
+      <c r="G19" s="33" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" ht="28.8" x14ac:dyDescent="0.25">
       <c r="B20" s="18"/>
       <c r="C20" s="19"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="33"/>
+      <c r="D20" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="E20" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="F20" s="20">
+        <v>46020</v>
+      </c>
+      <c r="G20" s="33" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B21" s="18"/>
       <c r="C21" s="19"/>
-      <c r="D21" s="14"/>
+      <c r="D21" s="14" t="s">
+        <v>85</v>
+      </c>
       <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="33"/>
-    </row>
-    <row r="22" spans="2:7" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="11"/>
-      <c r="C22" s="12"/>
-      <c r="D22" s="12"/>
-      <c r="E22" s="12"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="33"/>
+      <c r="F21" s="20">
+        <v>46020</v>
+      </c>
+      <c r="G21" s="33" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" ht="144" x14ac:dyDescent="0.25">
+      <c r="B22" s="18"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="38" t="s">
+        <v>88</v>
+      </c>
+      <c r="E22" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="F22" s="20">
+        <v>46020</v>
+      </c>
+      <c r="G22" s="33" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="11"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="13"/>
+      <c r="G23" s="33"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -2340,8 +2739,8 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CAC97C2-8F2F-4876-9208-CADAE372E0B5}">
-  <dimension ref="B3:F4"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <dimension ref="B3:F5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="47.33203125" customWidth="1"/>
     <col min="5" max="5" width="40.44140625" customWidth="1"/>
@@ -2367,6 +2766,11 @@
         <v>55</v>
       </c>
     </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="F5" t="s">
+        <v>64</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>